<commit_message>
fix(hardware): Update schematic pin alignment script and prototype BOM
</commit_message>
<xml_diff>
--- a/docs/Daneben_Hardware_BoM_Prototype.xlsx
+++ b/docs/Daneben_Hardware_BoM_Prototype.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/50d8e3b8d2fbeff0/Documents/Deutschland/HSNR/Studium/5.Semester/Mikro-contoller/Daneben Projekt/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_8A4398D7D06AC8AE6D55B0174E139E7B0DE58F6B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07BEE781-0D57-4052-9F6C-C7149436BA0F}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_8A43861F557B92EEE64D40F75B2F2E3E24098D65" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7595E73-91B6-4699-B4DB-EA5E88857AE3}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="74">
   <si>
     <t>DANEBEN! SMART IOT WASTE BIN SYSTEM — PROTOTYPE BILL OF MATERIALS (BOM)</t>
   </si>
@@ -71,7 +71,8 @@
 (Alt: €15.00)</t>
   </si>
   <si>
-    <t>Sense daughterboard with OV2640 camera (MPN: 113991115)</t>
+    <t>Sense daughterboard with OV2640 camera
+(MPN: 113991115)</t>
   </si>
   <si>
     <t>02</t>
@@ -270,12 +271,6 @@
   </si>
   <si>
     <t>Σ  TOTAL PROTOTYPE HARDWARE (GROSS INCL. 19% VAT)</t>
-  </si>
-  <si>
-    <t>Consolidated Sourcing</t>
-  </si>
-  <si>
-    <t>Master Prototype BoM</t>
   </si>
   <si>
     <t>16×</t>
@@ -360,14 +355,14 @@
       <name val="Segoe UI"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF64748B"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF15803D"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF64748B"/>
       <name val="Segoe UI"/>
     </font>
     <font>
@@ -445,7 +440,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -504,29 +499,26 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -846,26 +838,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
     </row>
     <row r="2" spans="1:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="3" spans="1:7" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:7" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1149,38 +1141,34 @@
         <v>69</v>
       </c>
       <c r="B16" s="27"/>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="F16" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="22" t="s">
+      <c r="G16" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="23" t="s">
+    </row>
+    <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="G16" s="21" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A16:D16"/>
     <mergeCell ref="A18:G18"/>
   </mergeCells>
   <printOptions gridLines="1"/>

</xml_diff>